<commit_message>
Colonne Lot (SPK / GO) dans le Gantt, l'XML et l'Excel
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_013W8KVJ4xCc6uDbxPYuViTn
</commit_message>
<xml_diff>
--- a/planning/Planning_EXE_15sem_Phase1_Decathlon_Campus_import_Excel.xlsx
+++ b/planning/Planning_EXE_15sem_Phase1_Decathlon_Campus_import_Excel.xlsx
@@ -855,7 +855,7 @@
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>VRD</t>
+          <t>GO</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
@@ -954,7 +954,7 @@
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>SPK/MOA</t>
+          <t>SPK</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
@@ -1079,7 +1079,7 @@
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>VRD</t>
+          <t>GO</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
@@ -1831,7 +1831,7 @@
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>GO/SPK</t>
+          <t>GO + SPK</t>
         </is>
       </c>
       <c r="G47" t="inlineStr">
@@ -2365,7 +2365,7 @@
       </c>
       <c r="F65" t="inlineStr">
         <is>
-          <t>VRD</t>
+          <t>GO</t>
         </is>
       </c>
       <c r="G65" t="inlineStr">
@@ -2398,7 +2398,7 @@
       </c>
       <c r="F66" t="inlineStr">
         <is>
-          <t>VRD</t>
+          <t>GO</t>
         </is>
       </c>
       <c r="G66" t="inlineStr">
@@ -2497,7 +2497,7 @@
       </c>
       <c r="F69" t="inlineStr">
         <is>
-          <t>VRD</t>
+          <t>GO</t>
         </is>
       </c>
       <c r="G69" t="inlineStr">
@@ -2543,7 +2543,7 @@
       </c>
       <c r="F71" t="inlineStr">
         <is>
-          <t>VRD</t>
+          <t>GO</t>
         </is>
       </c>
       <c r="G71" t="inlineStr">
@@ -2576,7 +2576,7 @@
       </c>
       <c r="F72" t="inlineStr">
         <is>
-          <t>VRD</t>
+          <t>GO</t>
         </is>
       </c>
       <c r="G72" t="inlineStr">
@@ -2675,7 +2675,7 @@
       </c>
       <c r="F75" t="inlineStr">
         <is>
-          <t>VRD</t>
+          <t>GO</t>
         </is>
       </c>
       <c r="G75" t="inlineStr">
@@ -2721,7 +2721,7 @@
       </c>
       <c r="F77" t="inlineStr">
         <is>
-          <t>VRD</t>
+          <t>GO</t>
         </is>
       </c>
       <c r="G77" t="inlineStr">
@@ -2754,7 +2754,7 @@
       </c>
       <c r="F78" t="inlineStr">
         <is>
-          <t>VRD</t>
+          <t>GO</t>
         </is>
       </c>
       <c r="G78" t="inlineStr">
@@ -2787,7 +2787,7 @@
       </c>
       <c r="F79" t="inlineStr">
         <is>
-          <t>VRD</t>
+          <t>GO</t>
         </is>
       </c>
       <c r="G79" t="inlineStr">
@@ -4983,7 +4983,7 @@
       </c>
       <c r="F151" t="inlineStr">
         <is>
-          <t>VRD</t>
+          <t>GO</t>
         </is>
       </c>
       <c r="G151" t="inlineStr">
@@ -5016,7 +5016,7 @@
       </c>
       <c r="F152" t="inlineStr">
         <is>
-          <t>VRD</t>
+          <t>GO</t>
         </is>
       </c>
       <c r="G152" t="inlineStr">
@@ -5049,7 +5049,7 @@
       </c>
       <c r="F153" t="inlineStr">
         <is>
-          <t>VRD</t>
+          <t>GO</t>
         </is>
       </c>
       <c r="G153" t="inlineStr">
@@ -5082,7 +5082,7 @@
       </c>
       <c r="F154" t="inlineStr">
         <is>
-          <t>VRD</t>
+          <t>GO</t>
         </is>
       </c>
       <c r="G154" t="inlineStr">
@@ -5115,7 +5115,7 @@
       </c>
       <c r="F155" t="inlineStr">
         <is>
-          <t>VRD</t>
+          <t>GO</t>
         </is>
       </c>
       <c r="G155" t="inlineStr">
@@ -5148,7 +5148,7 @@
       </c>
       <c r="F156" t="inlineStr">
         <is>
-          <t>VRD</t>
+          <t>GO</t>
         </is>
       </c>
       <c r="G156" t="inlineStr">
@@ -5181,7 +5181,7 @@
       </c>
       <c r="F157" t="inlineStr">
         <is>
-          <t>VRD</t>
+          <t>GO</t>
         </is>
       </c>
       <c r="G157" t="inlineStr">
@@ -5214,7 +5214,7 @@
       </c>
       <c r="F158" t="inlineStr">
         <is>
-          <t>VRD</t>
+          <t>GO</t>
         </is>
       </c>
       <c r="G158" t="inlineStr">

</xml_diff>

<commit_message>
Lot unique EIFFAGE (GO + VRD) dans planning, Gantt et exports
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_013W8KVJ4xCc6uDbxPYuViTn
</commit_message>
<xml_diff>
--- a/planning/Planning_EXE_15sem_Phase1_Decathlon_Campus_import_Excel.xlsx
+++ b/planning/Planning_EXE_15sem_Phase1_Decathlon_Campus_import_Excel.xlsx
@@ -550,7 +550,7 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>Limites de prestations 1 ; CCTP GO 5.1.3-5.1.5. Démarrage conditionné au dossier GN13.</t>
+          <t>Limites de prestations 1 ; CCTP EIFFAGE 5.1.3-5.1.5. Démarrage conditionné au dossier GN13.</t>
         </is>
       </c>
     </row>
@@ -616,7 +616,7 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>Limites de prestations 1 ; DPGF GO 5.1.6 (abonnements MOA). | Durée recalée EXE (15 semaines) : renfort d'équipes / travail en parallèle.</t>
+          <t>Limites de prestations 1 ; DPGF EIFFAGE 5.1.6 (abonnements MOA). | Durée recalée EXE (15 semaines) : renfort d'équipes / travail en parallèle.</t>
         </is>
       </c>
     </row>
@@ -695,7 +695,7 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>[GO] Pistes d'accès engins + plateforme de circulation sur géotextile classe 5</t>
+          <t>[EIFFAGE] Pistes d'accès engins + plateforme de circulation sur géotextile classe 5</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -710,12 +710,12 @@
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>GO</t>
+          <t>EIFFAGE</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>DPGF GO 5.3.3 ; Limites de prestations 1 (si nécessaire). | Durée recalée EXE (15 semaines) : renfort d'équipes / travail en parallèle.</t>
+          <t>DPGF EIFFAGE 5.3.3 ; Limites de prestations 1 (si nécessaire). | Durée recalée EXE (15 semaines) : renfort d'équipes / travail en parallèle.</t>
         </is>
       </c>
     </row>
@@ -728,7 +728,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>[GO] Dépose et stockage des bordures béton (réemploi en fin de chantier)</t>
+          <t>[EIFFAGE] Dépose et stockage des bordures béton (réemploi en fin de chantier)</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -743,12 +743,12 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>GO</t>
+          <t>EIFFAGE</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>DPGF GO 5.3.4.</t>
+          <t>DPGF EIFFAGE 5.3.4.</t>
         </is>
       </c>
     </row>
@@ -774,7 +774,7 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>[GO] Piquetage/marquage et reconnaissance des réseaux existants dans l'emprise (DN100 AEP, DN150 incendie, EU/EV/EP/électricité/fibre)</t>
+          <t>[EIFFAGE] Piquetage/marquage et reconnaissance des réseaux existants dans l'emprise (DN100 AEP, DN150 incendie, EU/EV/EP/électricité/fibre)</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -789,12 +789,12 @@
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>GO</t>
+          <t>EIFFAGE</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>CCTP GO 5.6.2 ; Limites de prestations 1. | Durée recalée EXE (15 semaines) : renfort d'équipes / travail en parallèle.</t>
+          <t>CCTP EIFFAGE 5.6.2 ; Limites de prestations 1. | Durée recalée EXE (15 semaines) : renfort d'équipes / travail en parallèle.</t>
         </is>
       </c>
     </row>
@@ -807,7 +807,7 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>[GO] Dévoiement réseau incendie DN150 + alimentation AEP/arrosage DN100 hors emprise radier (essais, DOE)</t>
+          <t>[EIFFAGE] Dévoiement réseau incendie DN150 + alimentation AEP/arrosage DN100 hors emprise radier (essais, DOE)</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -822,12 +822,12 @@
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>GO</t>
+          <t>EIFFAGE</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>DPGF GO 5.6.2 ; Limites de prestations 1. Continuité du réseau incendie à maintenir (coupure ponctuelle validée MOA). | Durée recalée EXE (15 semaines) : renfort d'équipes / travail en parallèle.</t>
+          <t>DPGF EIFFAGE 5.6.2 ; Limites de prestations 1. Continuité du réseau incendie à maintenir (coupure ponctuelle validée MOA). | Durée recalée EXE (15 semaines) : renfort d'équipes / travail en parallèle.</t>
         </is>
       </c>
     </row>
@@ -840,7 +840,7 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>[VRD] Dévoiement EU / EV / EP / électricité / fibre / arrosage si nécessaire (relevé NCA)</t>
+          <t>[EIFFAGE] Dévoiement EU / EV / EP / électricité / fibre / arrosage si nécessaire (relevé NCA)</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
@@ -855,7 +855,7 @@
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>GO</t>
+          <t>EIFFAGE</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
@@ -998,7 +998,7 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>[GO] Dépose brise-vue bois + charpente métallique support + grille d'accès/porte grillagée (évacuation)</t>
+          <t>[EIFFAGE] Dépose brise-vue bois + charpente métallique support + grille d'accès/porte grillagée (évacuation)</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
@@ -1013,12 +1013,12 @@
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>GO</t>
+          <t>EIFFAGE</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>DPGF GO 5.4.1 ; Limites de prestations 4 / Travaux réserves d'eau B2. Fait avant la vidange pour réduire l'indisponibilité. | Durée recalée EXE (15 semaines) : renfort d'équipes / travail en parallèle.</t>
+          <t>DPGF EIFFAGE 5.4.1 ; Limites de prestations 4 / Travaux réserves d'eau B2. Fait avant la vidange pour réduire l'indisponibilité. | Durée recalée EXE (15 semaines) : renfort d'équipes / travail en parallèle.</t>
         </is>
       </c>
     </row>
@@ -1051,7 +1051,7 @@
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>DPGF SPK 3.5 ; CCTP GO 5.4.2 (par lot SPK). Durée estimée (cuve acier 405 m³). | Durée recalée EXE (15 semaines) : renfort d'équipes / travail en parallèle.</t>
+          <t>DPGF SPK 3.5 ; CCTP EIFFAGE 5.4.2 (par lot SPK). Durée estimée (cuve acier 405 m³). | Durée recalée EXE (15 semaines) : renfort d'équipes / travail en parallèle.</t>
         </is>
       </c>
     </row>
@@ -1064,7 +1064,7 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>[VRD] Dépose des réseaux existants cuve B2 → local B2 → local A/GE (terrassement, évacuation, remblaiement)</t>
+          <t>[EIFFAGE] Dépose des réseaux existants cuve B2 → local B2 → local A/GE (terrassement, évacuation, remblaiement)</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
@@ -1079,12 +1079,12 @@
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>GO</t>
+          <t>EIFFAGE</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>DPGF GO 5.6.3 ; Limites de prestations 1 (dépose réseaux depuis cuve B2 jusqu'au local source A et B2 = VRD). | Durée recalée EXE (15 semaines) : renfort d'équipes / travail en parallèle.</t>
+          <t>DPGF EIFFAGE 5.6.3 ; Limites de prestations 1 (dépose réseaux depuis cuve B2 jusqu'au local source A et B2 = EIFFAGE). | Durée recalée EXE (15 semaines) : renfort d'équipes / travail en parallèle.</t>
         </is>
       </c>
     </row>
@@ -1097,7 +1097,7 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>[GO] Démolition du radier existant + évacuation des gravats (maîtrise poussières)</t>
+          <t>[EIFFAGE] Démolition du radier existant + évacuation des gravats (maîtrise poussières)</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
@@ -1112,12 +1112,12 @@
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>GO</t>
+          <t>EIFFAGE</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>DPGF GO 5.4.3 (ens.). Durée estimée. | Durée recalée EXE (15 semaines) : renfort d'équipes / travail en parallèle.</t>
+          <t>DPGF EIFFAGE 5.4.3 (ens.). Durée estimée. | Durée recalée EXE (15 semaines) : renfort d'équipes / travail en parallèle.</t>
         </is>
       </c>
     </row>
@@ -1130,7 +1130,7 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>[GO] Étêtage des fondations existantes à -1,00 m du niveau plateforme + évacuation</t>
+          <t>[EIFFAGE] Étêtage des fondations existantes à -1,00 m du niveau plateforme + évacuation</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
@@ -1145,7 +1145,7 @@
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>GO</t>
+          <t>EIFFAGE</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
@@ -1163,7 +1163,7 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>[GO] Relevé géomètre + plan de récolement des ouvrages enterrés, adaptation des fondations</t>
+          <t>[EIFFAGE] Relevé géomètre + plan de récolement des ouvrages enterrés, adaptation des fondations</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
@@ -1178,12 +1178,12 @@
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>GO</t>
+          <t>EIFFAGE</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>Limites de prestations 4 ; CCTP GO 5.4.4. | Durée recalée EXE (15 semaines) : renfort d'équipes / travail en parallèle.</t>
+          <t>Limites de prestations 4 ; CCTP EIFFAGE 5.4.4. | Durée recalée EXE (15 semaines) : renfort d'équipes / travail en parallèle.</t>
         </is>
       </c>
     </row>
@@ -1196,7 +1196,7 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>[GO] (OPTION 5.4.4) Purge des fondations profondes existantes (-80 cm sous niveau final) + remblai sablo-graveleux</t>
+          <t>[EIFFAGE] (OPTION 5.4.4) Purge des fondations profondes existantes (-80 cm sous niveau final) + remblai sablo-graveleux</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
@@ -1211,12 +1211,12 @@
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>GO</t>
+          <t>EIFFAGE</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>DPGF GO 5.4.4 OPTIONNEL : mode de fondation existant inconnu. Mettre la durée à 0 si l'option n'est pas retenue. | Durée recalée EXE (15 semaines) : renfort d'équipes / travail en parallèle.</t>
+          <t>DPGF EIFFAGE 5.4.4 OPTIONNEL : mode de fondation existant inconnu. Mettre la durée à 0 si l'option n'est pas retenue. | Durée recalée EXE (15 semaines) : renfort d'équipes / travail en parallèle.</t>
         </is>
       </c>
     </row>
@@ -1308,7 +1308,7 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>[GO] Dépose des pièces de scellement existantes local B2 + reprise des percements (DN300, DN200, DN150, échappement)</t>
+          <t>[EIFFAGE] Dépose des pièces de scellement existantes local B2 + reprise des percements (DN300, DN200, DN150, échappement)</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
@@ -1323,12 +1323,12 @@
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>GO</t>
+          <t>EIFFAGE</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>DPGF GO 5.8.2 ; Limites de prestations Travaux source B2. | Durée recalée EXE (15 semaines) : renfort d'équipes / travail en parallèle.</t>
+          <t>DPGF EIFFAGE 5.8.2 ; Limites de prestations Travaux source B2. | Durée recalée EXE (15 semaines) : renfort d'équipes / travail en parallèle.</t>
         </is>
       </c>
     </row>
@@ -1341,7 +1341,7 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>[GO] Démolition contrôlée réservation dalle basse et soubassement local GE (sciage, mise à nu des armatures)</t>
+          <t>[EIFFAGE] Démolition contrôlée réservation dalle basse et soubassement local GE (sciage, mise à nu des armatures)</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
@@ -1356,12 +1356,12 @@
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>GO</t>
+          <t>EIFFAGE</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>DPGF GO 5.8.5 ; Limites de prestations Travaux local GE. | Durée recalée EXE (15 semaines) : renfort d'équipes / travail en parallèle.</t>
+          <t>DPGF EIFFAGE 5.8.5 ; Limites de prestations Travaux local GE. | Durée recalée EXE (15 semaines) : renfort d'équipes / travail en parallèle.</t>
         </is>
       </c>
     </row>
@@ -1374,7 +1374,7 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>[GO] Dépose pièce de scellement existante local GE + création du percement DN200</t>
+          <t>[EIFFAGE] Dépose pièce de scellement existante local GE + création du percement DN200</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
@@ -1389,7 +1389,7 @@
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>GO</t>
+          <t>EIFFAGE</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
@@ -1420,7 +1420,7 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>[GO] Plateforme de travail pour pieux (portance EV2 &gt; 50 MPa, géotextile)</t>
+          <t>[EIFFAGE] Plateforme de travail pour pieux (portance EV2 &gt; 50 MPa, géotextile)</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
@@ -1435,12 +1435,12 @@
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>GO</t>
+          <t>EIFFAGE</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>Limites de prestations 4 ; DPGF GO 5.3.3. | Durée recalée EXE (15 semaines) : renfort d'équipes / travail en parallèle.</t>
+          <t>Limites de prestations 4 ; DPGF EIFFAGE 5.3.3. | Durée recalée EXE (15 semaines) : renfort d'équipes / travail en parallèle.</t>
         </is>
       </c>
     </row>
@@ -1453,7 +1453,7 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>[GO] Épuisement des eaux / rabattement de nappe (nappe ~ 27,4 NGF) pendant les fondations</t>
+          <t>[EIFFAGE] Épuisement des eaux / rabattement de nappe (nappe ~ 27,4 NGF) pendant les fondations</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
@@ -1468,12 +1468,12 @@
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>GO</t>
+          <t>EIFFAGE</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>DPGF GO 5.3.7 ; CCTP GO 4.7.2 ; Limites de prestations 3. Hamac plateforme → coulage radier.</t>
+          <t>DPGF EIFFAGE 5.3.7 ; CCTP EIFFAGE 4.7.2 ; Limites de prestations 3. Hamac plateforme → coulage radier.</t>
         </is>
       </c>
     </row>
@@ -1486,7 +1486,7 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>[GO] Pieux à tarière creuse (amenée/repli du matériel, forage, armatures, béton) - ~20 à 25 u. à confirmer PEO</t>
+          <t>[EIFFAGE] Pieux à tarière creuse (amenée/repli du matériel, forage, armatures, béton) - ~20 à 25 u. à confirmer PEO</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
@@ -1501,12 +1501,12 @@
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>GO</t>
+          <t>EIFFAGE</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>DPGF GO 5.5.1 (u) ; CCTP GO 5.5.1 ; G2PRO Fondasol. Hypothèse ~5 pieux/jour. | Durée recalée EXE (15 semaines) : renfort d'équipes / travail en parallèle.</t>
+          <t>DPGF EIFFAGE 5.5.1 (u) ; CCTP EIFFAGE 5.5.1 ; G2PRO Fondasol. Hypothèse ~5 pieux/jour. | Durée recalée EXE (15 semaines) : renfort d'équipes / travail en parallèle.</t>
         </is>
       </c>
     </row>
@@ -1519,7 +1519,7 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>[GO] Stockage sur polyane et évacuation des terres et boues de forage + nettoyage voies</t>
+          <t>[EIFFAGE] Stockage sur polyane et évacuation des terres et boues de forage + nettoyage voies</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
@@ -1534,12 +1534,12 @@
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>GO</t>
+          <t>EIFFAGE</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>DPGF GO 5.5.2 / 5.3.8. | Durée recalée EXE (15 semaines) : renfort d'équipes / travail en parallèle.</t>
+          <t>DPGF EIFFAGE 5.5.2 / 5.3.8. | Durée recalée EXE (15 semaines) : renfort d'équipes / travail en parallèle.</t>
         </is>
       </c>
     </row>
@@ -1552,7 +1552,7 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>[GO] Essais et contrôle des pieux (DTU 13.2 / NF P94-262)</t>
+          <t>[EIFFAGE] Essais et contrôle des pieux (DTU 13.2 / NF P94-262)</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
@@ -1567,12 +1567,12 @@
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>GO</t>
+          <t>EIFFAGE</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>CCTP GO 5.5.1.</t>
+          <t>CCTP EIFFAGE 5.5.1.</t>
         </is>
       </c>
     </row>
@@ -1585,7 +1585,7 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>[GO] Recépage des pieux</t>
+          <t>[EIFFAGE] Recépage des pieux</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
@@ -1600,12 +1600,12 @@
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>GO</t>
+          <t>EIFFAGE</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>CCTP GO 5.5.1. | Durée recalée EXE (15 semaines) : renfort d'équipes / travail en parallèle.</t>
+          <t>CCTP EIFFAGE 5.5.1. | Durée recalée EXE (15 semaines) : renfort d'équipes / travail en parallèle.</t>
         </is>
       </c>
     </row>
@@ -1618,7 +1618,7 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>[GO] Terrassement fouille radier + substitution remblais de portance + fond de forme (débord 1 m)</t>
+          <t>[EIFFAGE] Terrassement fouille radier + substitution remblais de portance + fond de forme (débord 1 m)</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
@@ -1633,12 +1633,12 @@
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>GO</t>
+          <t>EIFFAGE</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>DPGF GO 5.3.5 / 5.3.6 (m³). | Durée recalée EXE (15 semaines) : renfort d'équipes / travail en parallèle.</t>
+          <t>DPGF EIFFAGE 5.3.5 / 5.3.6 (m³). | Durée recalée EXE (15 semaines) : renfort d'équipes / travail en parallèle.</t>
         </is>
       </c>
     </row>
@@ -1651,7 +1651,7 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>[GO] Puisard de trop-plein de la cuve (terrassement, béton de propreté, grille circulable)</t>
+          <t>[EIFFAGE] Puisard de trop-plein de la cuve (terrassement, béton de propreté, grille circulable)</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
@@ -1666,12 +1666,12 @@
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>GO</t>
+          <t>EIFFAGE</t>
         </is>
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>DPGF GO 5.6.6 ; CCTP GO 5.6.6. | Durée recalée EXE (15 semaines) : renfort d'équipes / travail en parallèle.</t>
+          <t>DPGF EIFFAGE 5.6.6 ; CCTP EIFFAGE 5.6.6. | Durée recalée EXE (15 semaines) : renfort d'équipes / travail en parallèle.</t>
         </is>
       </c>
     </row>
@@ -1684,7 +1684,7 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>[GO] Béton de propreté (e &gt;= 5 cm) sous radier</t>
+          <t>[EIFFAGE] Béton de propreté (e &gt;= 5 cm) sous radier</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
@@ -1699,12 +1699,12 @@
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>GO</t>
+          <t>EIFFAGE</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>DPGF GO 5.5.3.</t>
+          <t>DPGF EIFFAGE 5.5.3.</t>
         </is>
       </c>
     </row>
@@ -1717,7 +1717,7 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>[GO] Boucle de terre fond de fouille (câble nu 25 mm2, R &lt;= 3 ohms) + attentes de terre cuve</t>
+          <t>[EIFFAGE] Boucle de terre fond de fouille (câble nu 25 mm2, R &lt;= 3 ohms) + attentes de terre cuve</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
@@ -1732,12 +1732,12 @@
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>GO</t>
+          <t>EIFFAGE</t>
         </is>
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>DPGF GO 5.3.9 ; Limites de prestations 3 (boucle de terre du radier = GO). | Durée recalée EXE (15 semaines) : renfort d'équipes / travail en parallèle.</t>
+          <t>DPGF EIFFAGE 5.3.9 ; Limites de prestations 3 (boucle de terre du radier = EIFFAGE). | Durée recalée EXE (15 semaines) : renfort d'équipes / travail en parallèle.</t>
         </is>
       </c>
     </row>
@@ -1750,7 +1750,7 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>[GO] Pose massifs, platines et boîtes de réservation de pre-scellement (poteaux brise-vue)</t>
+          <t>[EIFFAGE] Pose massifs, platines et boîtes de réservation de pre-scellement (poteaux brise-vue)</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
@@ -1765,12 +1765,12 @@
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>GO</t>
+          <t>EIFFAGE</t>
         </is>
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>DPGF GO 5.5.4. | Durée recalée EXE (15 semaines) : renfort d'équipes / travail en parallèle.</t>
+          <t>DPGF EIFFAGE 5.5.4. | Durée recalée EXE (15 semaines) : renfort d'équipes / travail en parallèle.</t>
         </is>
       </c>
     </row>
@@ -1783,7 +1783,7 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>[GO] Couche de forme + sablon d'égalisation + film polyéthylène</t>
+          <t>[EIFFAGE] Couche de forme + sablon d'égalisation + film polyéthylène</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
@@ -1798,12 +1798,12 @@
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>GO</t>
+          <t>EIFFAGE</t>
         </is>
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t>CCTP GO 5.5.5. | Durée recalée EXE (15 semaines) : renfort d'équipes / travail en parallèle.</t>
+          <t>CCTP EIFFAGE 5.5.5. | Durée recalée EXE (15 semaines) : renfort d'équipes / travail en parallèle.</t>
         </is>
       </c>
     </row>
@@ -1816,7 +1816,7 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>[GO] Pose et incorporation de la tuyauterie d'aspiration DN300 sous radier (fournie SPK) + validation implantation SPK/GO</t>
+          <t>[EIFFAGE] Pose et incorporation de la tuyauterie d'aspiration DN300 sous radier (fournie SPK) + validation implantation SPK/EIFFAGE</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
@@ -1831,12 +1831,12 @@
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>GO + SPK</t>
+          <t>EIFFAGE + SPK</t>
         </is>
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t>Limites de prestations 4 : GO réalise, SPK accompagne (P) et valide l'implantation avant coulée. | Durée recalée EXE (15 semaines) : renfort d'équipes / travail en parallèle.</t>
+          <t>Limites de prestations 4 : EIFFAGE réalise, SPK accompagne (P) et valide l'implantation avant coulée. | Durée recalée EXE (15 semaines) : renfort d'équipes / travail en parallèle.</t>
         </is>
       </c>
     </row>
@@ -1849,7 +1849,7 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>[GO] Drain périphérique / gestion des eaux autour du radier (si G2PRO l'impose)</t>
+          <t>[EIFFAGE] Drain périphérique / gestion des eaux autour du radier (si G2PRO l'impose)</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
@@ -1864,7 +1864,7 @@
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>GO</t>
+          <t>EIFFAGE</t>
         </is>
       </c>
       <c r="G48" t="inlineStr">
@@ -1882,7 +1882,7 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>[GO] Ferraillage radier (TS + HA), attentes pieux, réservations, fourreaux, coffrage de rives et bêches périphériques</t>
+          <t>[EIFFAGE] Ferraillage radier (TS + HA), attentes pieux, réservations, fourreaux, coffrage de rives et bêches périphériques</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
@@ -1897,12 +1897,12 @@
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>GO</t>
+          <t>EIFFAGE</t>
         </is>
       </c>
       <c r="G49" t="inlineStr">
         <is>
-          <t>DPGF GO 5.5.5 (m³). Durée estimée (radier ~ Ø 14 m). | Durée recalée EXE (15 semaines) : renfort d'équipes / travail en parallèle.</t>
+          <t>DPGF EIFFAGE 5.5.5 (m³). Durée estimée (radier ~ Ø 14 m). | Durée recalée EXE (15 semaines) : renfort d'équipes / travail en parallèle.</t>
         </is>
       </c>
     </row>
@@ -1915,7 +1915,7 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>[GO] Coulage du radier béton C25/30 XC2 XF1 (parement soigné, circulations brossées antidérapantes)</t>
+          <t>[EIFFAGE] Coulage du radier béton C25/30 XC2 XF1 (parement soigné, circulations brossées antidérapantes)</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
@@ -1930,12 +1930,12 @@
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t>GO</t>
+          <t>EIFFAGE</t>
         </is>
       </c>
       <c r="G50" t="inlineStr">
         <is>
-          <t>DPGF GO 5.5.5 ; CCTP GO 4.4.</t>
+          <t>DPGF EIFFAGE 5.5.5 ; CCTP EIFFAGE 4.4.</t>
         </is>
       </c>
     </row>
@@ -1948,7 +1948,7 @@
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>[GO] Durcissement du radier avant chargement de la cuve (délai à valider BET / bureau de contrôle)</t>
+          <t>[EIFFAGE] Durcissement du radier avant chargement de la cuve (délai à valider BET / bureau de contrôle)</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
@@ -1963,7 +1963,7 @@
       </c>
       <c r="F51" t="inlineStr">
         <is>
-          <t>GO</t>
+          <t>EIFFAGE</t>
         </is>
       </c>
       <c r="G51" t="inlineStr">
@@ -2192,7 +2192,7 @@
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>[GO] Joint ciment périphérique autour de la cornière de fixation de la cuve</t>
+          <t>[EIFFAGE] Joint ciment périphérique autour de la cornière de fixation de la cuve</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
@@ -2207,12 +2207,12 @@
       </c>
       <c r="F59" t="inlineStr">
         <is>
-          <t>GO</t>
+          <t>EIFFAGE</t>
         </is>
       </c>
       <c r="G59" t="inlineStr">
         <is>
-          <t>DPGF GO 5.8.1 (ml) ; Limites de prestations 4.</t>
+          <t>DPGF EIFFAGE 5.8.1 (ml) ; Limites de prestations 4.</t>
         </is>
       </c>
     </row>
@@ -2350,7 +2350,7 @@
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>[VRD] Ouverture tranchée commune (~ 25 ml estimés)</t>
+          <t>[EIFFAGE] Ouverture tranchée commune (~ 25 ml estimés)</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
@@ -2365,12 +2365,12 @@
       </c>
       <c r="F65" t="inlineStr">
         <is>
-          <t>GO</t>
+          <t>EIFFAGE</t>
         </is>
       </c>
       <c r="G65" t="inlineStr">
         <is>
-          <t>DPGF GO 5.6.1 (ml) ; Limites de prestations 5. Longueur estimée : à relever sur plan. | Durée recalée EXE (15 semaines) : renfort d'équipes / travail en parallèle.</t>
+          <t>DPGF EIFFAGE 5.6.1 (ml) ; Limites de prestations 5. Longueur estimée : à relever sur plan. | Durée recalée EXE (15 semaines) : renfort d'équipes / travail en parallèle.</t>
         </is>
       </c>
     </row>
@@ -2383,7 +2383,7 @@
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>[VRD] Fourreaux électriques 2 x Ø90 (local B2 / réserve d'eau) + chambre de tirage</t>
+          <t>[EIFFAGE] Fourreaux électriques 2 x Ø90 (local B2 / réserve d'eau) + chambre de tirage</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
@@ -2398,12 +2398,12 @@
       </c>
       <c r="F66" t="inlineStr">
         <is>
-          <t>GO</t>
+          <t>EIFFAGE</t>
         </is>
       </c>
       <c r="G66" t="inlineStr">
         <is>
-          <t>DPGF GO 5.6.4 / 5.6.5 ; Limites de prestations 5 (Électricité). | Durée recalée EXE (15 semaines) : renfort d'équipes / travail en parallèle.</t>
+          <t>DPGF EIFFAGE 5.6.4 / 5.6.5 ; Limites de prestations 5 (Électricité). | Durée recalée EXE (15 semaines) : renfort d'équipes / travail en parallèle.</t>
         </is>
       </c>
     </row>
@@ -2482,7 +2482,7 @@
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>[VRD] Grillage avertisseur + remblaiement et compactage tranchée 1 (95 % OPM)</t>
+          <t>[EIFFAGE] Grillage avertisseur + remblaiement et compactage tranchée 1 (95 % OPM)</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
@@ -2497,12 +2497,12 @@
       </c>
       <c r="F69" t="inlineStr">
         <is>
-          <t>GO</t>
+          <t>EIFFAGE</t>
         </is>
       </c>
       <c r="G69" t="inlineStr">
         <is>
-          <t>Limites de prestations 5 : remblaiement VRD après pose SPK.</t>
+          <t>Limites de prestations 5 : remblaiement EIFFAGE après pose SPK.</t>
         </is>
       </c>
     </row>
@@ -2528,7 +2528,7 @@
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>[VRD] Ouverture tranchée commune (~ 60 ml estimés, sciage voirie lourde + espace vert)</t>
+          <t>[EIFFAGE] Ouverture tranchée commune (~ 60 ml estimés, sciage voirie lourde + espace vert)</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
@@ -2543,12 +2543,12 @@
       </c>
       <c r="F71" t="inlineStr">
         <is>
-          <t>GO</t>
+          <t>EIFFAGE</t>
         </is>
       </c>
       <c r="G71" t="inlineStr">
         <is>
-          <t>DPGF GO 5.6.1 / 5.3.2 ; Limites de prestations 5. Longueur estimée. | Durée recalée EXE (15 semaines) : renfort d'équipes / travail en parallèle.</t>
+          <t>DPGF EIFFAGE 5.6.1 / 5.3.2 ; Limites de prestations 5. Longueur estimée. | Durée recalée EXE (15 semaines) : renfort d'équipes / travail en parallèle.</t>
         </is>
       </c>
     </row>
@@ -2561,7 +2561,7 @@
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>[VRD] Fourreaux électriques 2 x Ø90 (local GE / local B2) + chambre de tirage</t>
+          <t>[EIFFAGE] Fourreaux électriques 2 x Ø90 (local GE / local B2) + chambre de tirage</t>
         </is>
       </c>
       <c r="D72" t="inlineStr">
@@ -2576,12 +2576,12 @@
       </c>
       <c r="F72" t="inlineStr">
         <is>
-          <t>GO</t>
+          <t>EIFFAGE</t>
         </is>
       </c>
       <c r="G72" t="inlineStr">
         <is>
-          <t>DPGF GO 5.6.4 / 5.6.5. | Durée recalée EXE (15 semaines) : renfort d'équipes / travail en parallèle.</t>
+          <t>DPGF EIFFAGE 5.6.4 / 5.6.5. | Durée recalée EXE (15 semaines) : renfort d'équipes / travail en parallèle.</t>
         </is>
       </c>
     </row>
@@ -2660,7 +2660,7 @@
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>[VRD] Grillage avertisseur + remblaiement et compactage tranchée 2</t>
+          <t>[EIFFAGE] Grillage avertisseur + remblaiement et compactage tranchée 2</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
@@ -2675,7 +2675,7 @@
       </c>
       <c r="F75" t="inlineStr">
         <is>
-          <t>GO</t>
+          <t>EIFFAGE</t>
         </is>
       </c>
       <c r="G75" t="inlineStr">
@@ -2706,7 +2706,7 @@
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>[VRD] Tranchée + réseau de collecte extérieur EU PVC DN200 (puisard/vidange → regard existant), regard 500x500</t>
+          <t>[EIFFAGE] Tranchée + réseau de collecte extérieur EU PVC DN200 (puisard/vidange → regard existant), regard 500x500</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
@@ -2721,12 +2721,12 @@
       </c>
       <c r="F77" t="inlineStr">
         <is>
-          <t>GO</t>
+          <t>EIFFAGE</t>
         </is>
       </c>
       <c r="G77" t="inlineStr">
         <is>
-          <t>DPGF GO 5.6.7 (ml) ; Limites de prestations 5. | Durée recalée EXE (15 semaines) : renfort d'équipes / travail en parallèle.</t>
+          <t>DPGF EIFFAGE 5.6.7 (ml) ; Limites de prestations 5. | Durée recalée EXE (15 semaines) : renfort d'équipes / travail en parallèle.</t>
         </is>
       </c>
     </row>
@@ -2739,7 +2739,7 @@
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>[VRD] Raccordement sur réseau EU existant (branchement), boîte de branchement, reprise des sorties EU à 1,00 m</t>
+          <t>[EIFFAGE] Raccordement sur réseau EU existant (branchement), boîte de branchement, reprise des sorties EU à 1,00 m</t>
         </is>
       </c>
       <c r="D78" t="inlineStr">
@@ -2754,7 +2754,7 @@
       </c>
       <c r="F78" t="inlineStr">
         <is>
-          <t>GO</t>
+          <t>EIFFAGE</t>
         </is>
       </c>
       <c r="G78" t="inlineStr">
@@ -2772,7 +2772,7 @@
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>[VRD] Remblaiement et compactage tranchée EU</t>
+          <t>[EIFFAGE] Remblaiement et compactage tranchée EU</t>
         </is>
       </c>
       <c r="D79" t="inlineStr">
@@ -2787,7 +2787,7 @@
       </c>
       <c r="F79" t="inlineStr">
         <is>
-          <t>GO</t>
+          <t>EIFFAGE</t>
         </is>
       </c>
       <c r="G79" t="inlineStr">
@@ -2864,7 +2864,7 @@
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>[GO] Pose nouvelles pièces de scellement local B2 (DN300, DN200, DN150, échappement), reprise mortier, étanchéité, calfeutrement</t>
+          <t>[EIFFAGE] Pose nouvelles pièces de scellement local B2 (DN300, DN200, DN150, échappement), reprise mortier, étanchéité, calfeutrement</t>
         </is>
       </c>
       <c r="D83" t="inlineStr">
@@ -2879,12 +2879,12 @@
       </c>
       <c r="F83" t="inlineStr">
         <is>
-          <t>GO</t>
+          <t>EIFFAGE</t>
         </is>
       </c>
       <c r="G83" t="inlineStr">
         <is>
-          <t>DPGF GO 5.8.3 ; Limites de prestations Travaux source B2. | Durée recalée EXE (15 semaines) : renfort d'équipes / travail en parallèle.</t>
+          <t>DPGF EIFFAGE 5.8.3 ; Limites de prestations Travaux source B2. | Durée recalée EXE (15 semaines) : renfort d'équipes / travail en parallèle.</t>
         </is>
       </c>
     </row>
@@ -2897,7 +2897,7 @@
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>[GO] Pose nouvelle pièce de scellement refoulement DN200 local GE + calfeutrement</t>
+          <t>[EIFFAGE] Pose nouvelle pièce de scellement refoulement DN200 local GE + calfeutrement</t>
         </is>
       </c>
       <c r="D84" t="inlineStr">
@@ -2912,7 +2912,7 @@
       </c>
       <c r="F84" t="inlineStr">
         <is>
-          <t>GO</t>
+          <t>EIFFAGE</t>
         </is>
       </c>
       <c r="G84" t="inlineStr">
@@ -3194,7 +3194,7 @@
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>[GO] Restauration couche de forme, dalle portée, soubassement et cuvelage local GE + durcisseur de dalle</t>
+          <t>[EIFFAGE] Restauration couche de forme, dalle portée, soubassement et cuvelage local GE + durcisseur de dalle</t>
         </is>
       </c>
       <c r="D93" t="inlineStr">
@@ -3209,12 +3209,12 @@
       </c>
       <c r="F93" t="inlineStr">
         <is>
-          <t>GO</t>
+          <t>EIFFAGE</t>
         </is>
       </c>
       <c r="G93" t="inlineStr">
         <is>
-          <t>DPGF GO 5.8.5 ; Limites de prestations Travaux local GE. | Durée recalée EXE (15 semaines) : renfort d'équipes / travail en parallèle.</t>
+          <t>DPGF EIFFAGE 5.8.5 ; Limites de prestations Travaux local GE. | Durée recalée EXE (15 semaines) : renfort d'équipes / travail en parallèle.</t>
         </is>
       </c>
     </row>
@@ -3240,7 +3240,7 @@
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>[GO] Percement des voiles béton façade Nord : ventilation haute et basse + redressement des tableaux</t>
+          <t>[EIFFAGE] Percement des voiles béton façade Nord : ventilation haute et basse + redressement des tableaux</t>
         </is>
       </c>
       <c r="D95" t="inlineStr">
@@ -3255,12 +3255,12 @@
       </c>
       <c r="F95" t="inlineStr">
         <is>
-          <t>GO</t>
+          <t>EIFFAGE</t>
         </is>
       </c>
       <c r="G95" t="inlineStr">
         <is>
-          <t>DPGF GO 5.8.4 (m²) ; Limites de prestations Travaux local sprinkleur source A. | Durée recalée EXE (15 semaines) : renfort d'équipes / travail en parallèle.</t>
+          <t>DPGF EIFFAGE 5.8.4 (m²) ; Limites de prestations Travaux local sprinkleur source A. | Durée recalée EXE (15 semaines) : renfort d'équipes / travail en parallèle.</t>
         </is>
       </c>
     </row>
@@ -4823,7 +4823,7 @@
       </c>
       <c r="C146" t="inlineStr">
         <is>
-          <t>[GO/CM] Montage charpente métallique brise-vue (poteaux, pannes, contreventement) + scellement définitif des ancrages</t>
+          <t>[EIFFAGE] Montage charpente métallique brise-vue (poteaux, pannes, contreventement) + scellement définitif des ancrages</t>
         </is>
       </c>
       <c r="D146" t="inlineStr">
@@ -4838,12 +4838,12 @@
       </c>
       <c r="F146" t="inlineStr">
         <is>
-          <t>GO</t>
+          <t>EIFFAGE</t>
         </is>
       </c>
       <c r="G146" t="inlineStr">
         <is>
-          <t>DPGF GO 5.7.1 ; Limites de prestations 4. CCTP GO 1 : cuve et réseaux avant brise-vue. | Durée recalée EXE (15 semaines) : renfort d'équipes / travail en parallèle.</t>
+          <t>DPGF EIFFAGE 5.7.1 ; Limites de prestations 4. CCTP EIFFAGE 1 : cuve et réseaux avant brise-vue. | Durée recalée EXE (15 semaines) : renfort d'équipes / travail en parallèle.</t>
         </is>
       </c>
     </row>
@@ -4856,7 +4856,7 @@
       </c>
       <c r="C147" t="inlineStr">
         <is>
-          <t>[GO/Bardage] Sous-construction du bardage (profils oméga acier galvanisé sur poteaux)</t>
+          <t>[EIFFAGE] Sous-construction du bardage (profils oméga acier galvanisé sur poteaux)</t>
         </is>
       </c>
       <c r="D147" t="inlineStr">
@@ -4871,12 +4871,12 @@
       </c>
       <c r="F147" t="inlineStr">
         <is>
-          <t>GO</t>
+          <t>EIFFAGE</t>
         </is>
       </c>
       <c r="G147" t="inlineStr">
         <is>
-          <t>DPGF GO 5.9.1 (m²). Durée estimée. | Durée recalée EXE (15 semaines) : renfort d'équipes / travail en parallèle.</t>
+          <t>DPGF EIFFAGE 5.9.1 (m²). Durée estimée. | Durée recalée EXE (15 semaines) : renfort d'équipes / travail en parallèle.</t>
         </is>
       </c>
     </row>
@@ -4889,7 +4889,7 @@
       </c>
       <c r="C148" t="inlineStr">
         <is>
-          <t>[GO/Bardage] Lames de bardage bois douglas à claire-voie (espacement 20 mm), coupes à 45°, saturateur</t>
+          <t>[EIFFAGE] Lames de bardage bois douglas à claire-voie (espacement 20 mm), coupes à 45°, saturateur</t>
         </is>
       </c>
       <c r="D148" t="inlineStr">
@@ -4904,12 +4904,12 @@
       </c>
       <c r="F148" t="inlineStr">
         <is>
-          <t>GO</t>
+          <t>EIFFAGE</t>
         </is>
       </c>
       <c r="G148" t="inlineStr">
         <is>
-          <t>DPGF GO 5.9.2 (m²). Hypothèse ~40 m²/jour. | Durée recalée EXE (15 semaines) : renfort d'équipes / travail en parallèle.</t>
+          <t>DPGF EIFFAGE 5.9.2 (m²). Hypothèse ~40 m²/jour. | Durée recalée EXE (15 semaines) : renfort d'équipes / travail en parallèle.</t>
         </is>
       </c>
     </row>
@@ -4922,7 +4922,7 @@
       </c>
       <c r="C149" t="inlineStr">
         <is>
-          <t>[GO] Pose porte d'accès cuve B2 (ferme-porte, barre anti-panique, serrure compatible site)</t>
+          <t>[EIFFAGE] Pose porte d'accès cuve B2 (ferme-porte, barre anti-panique, serrure compatible site)</t>
         </is>
       </c>
       <c r="D149" t="inlineStr">
@@ -4937,12 +4937,12 @@
       </c>
       <c r="F149" t="inlineStr">
         <is>
-          <t>GO</t>
+          <t>EIFFAGE</t>
         </is>
       </c>
       <c r="G149" t="inlineStr">
         <is>
-          <t>DPGF GO 5.9.3.</t>
+          <t>DPGF EIFFAGE 5.9.3.</t>
         </is>
       </c>
     </row>
@@ -4955,7 +4955,7 @@
       </c>
       <c r="C150" t="inlineStr">
         <is>
-          <t>15. VOIRIES ET ESPACES VERTS - REMISE EN ÉTAT (VRD)</t>
+          <t>15. VOIRIES ET ESPACES VERTS - REMISE EN ÉTAT (EIFFAGE)</t>
         </is>
       </c>
     </row>
@@ -4968,7 +4968,7 @@
       </c>
       <c r="C151" t="inlineStr">
         <is>
-          <t>[VRD] Remise en place des bordures béton (joints résistants UV et hydrocarbures)</t>
+          <t>[EIFFAGE] Remise en place des bordures béton (joints résistants UV et hydrocarbures)</t>
         </is>
       </c>
       <c r="D151" t="inlineStr">
@@ -4983,12 +4983,12 @@
       </c>
       <c r="F151" t="inlineStr">
         <is>
-          <t>GO</t>
+          <t>EIFFAGE</t>
         </is>
       </c>
       <c r="G151" t="inlineStr">
         <is>
-          <t>DPGF GO 5.10.3 (ml).</t>
+          <t>DPGF EIFFAGE 5.10.3 (ml).</t>
         </is>
       </c>
     </row>
@@ -5001,7 +5001,7 @@
       </c>
       <c r="C152" t="inlineStr">
         <is>
-          <t>[VRD] Réfection voie technique : reprofilage GNT 30 cm, géotextile cl.4, enrobé noir 5 cm au droit des réseaux</t>
+          <t>[EIFFAGE] Réfection voie technique : reprofilage GNT 30 cm, géotextile cl.4, enrobé noir 5 cm au droit des réseaux</t>
         </is>
       </c>
       <c r="D152" t="inlineStr">
@@ -5016,12 +5016,12 @@
       </c>
       <c r="F152" t="inlineStr">
         <is>
-          <t>GO</t>
+          <t>EIFFAGE</t>
         </is>
       </c>
       <c r="G152" t="inlineStr">
         <is>
-          <t>DPGF GO 5.10.4 (m²) ; Limites de prestations 6. | Durée recalée EXE (15 semaines) : renfort d'équipes / travail en parallèle.</t>
+          <t>DPGF EIFFAGE 5.10.4 (m²) ; Limites de prestations 6. | Durée recalée EXE (15 semaines) : renfort d'équipes / travail en parallèle.</t>
         </is>
       </c>
     </row>
@@ -5034,7 +5034,7 @@
       </c>
       <c r="C153" t="inlineStr">
         <is>
-          <t>[VRD] Dépose des pistes d'accès chantier + évacuation + reprofilage</t>
+          <t>[EIFFAGE] Dépose des pistes d'accès chantier + évacuation + reprofilage</t>
         </is>
       </c>
       <c r="D153" t="inlineStr">
@@ -5049,12 +5049,12 @@
       </c>
       <c r="F153" t="inlineStr">
         <is>
-          <t>GO</t>
+          <t>EIFFAGE</t>
         </is>
       </c>
       <c r="G153" t="inlineStr">
         <is>
-          <t>CCTP GO 5.3.3. | Durée recalée EXE (15 semaines) : renfort d'équipes / travail en parallèle.</t>
+          <t>CCTP EIFFAGE 5.3.3. | Durée recalée EXE (15 semaines) : renfort d'équipes / travail en parallèle.</t>
         </is>
       </c>
     </row>
@@ -5067,7 +5067,7 @@
       </c>
       <c r="C154" t="inlineStr">
         <is>
-          <t>[VRD] Mouvements de terres, nivellement espaces verts + apport terre végétale 0,30 m mini</t>
+          <t>[EIFFAGE] Mouvements de terres, nivellement espaces verts + apport terre végétale 0,30 m mini</t>
         </is>
       </c>
       <c r="D154" t="inlineStr">
@@ -5082,7 +5082,7 @@
       </c>
       <c r="F154" t="inlineStr">
         <is>
-          <t>GO</t>
+          <t>EIFFAGE</t>
         </is>
       </c>
       <c r="G154" t="inlineStr">
@@ -5100,7 +5100,7 @@
       </c>
       <c r="C155" t="inlineStr">
         <is>
-          <t>[VRD] Préparation avant engazonnement (nettoyage, rotavator 0,20 m, amendements, réglage)</t>
+          <t>[EIFFAGE] Préparation avant engazonnement (nettoyage, rotavator 0,20 m, amendements, réglage)</t>
         </is>
       </c>
       <c r="D155" t="inlineStr">
@@ -5115,12 +5115,12 @@
       </c>
       <c r="F155" t="inlineStr">
         <is>
-          <t>GO</t>
+          <t>EIFFAGE</t>
         </is>
       </c>
       <c r="G155" t="inlineStr">
         <is>
-          <t>DPGF GO 5.10.1. | Durée recalée EXE (15 semaines) : renfort d'équipes / travail en parallèle.</t>
+          <t>DPGF EIFFAGE 5.10.1. | Durée recalée EXE (15 semaines) : renfort d'équipes / travail en parallèle.</t>
         </is>
       </c>
     </row>
@@ -5133,7 +5133,7 @@
       </c>
       <c r="C156" t="inlineStr">
         <is>
-          <t>[VRD] Engazonnement (semis 3 kg/are, roulage, ratissage) - plantations gazon</t>
+          <t>[EIFFAGE] Engazonnement (semis 3 kg/are, roulage, ratissage) - plantations gazon</t>
         </is>
       </c>
       <c r="D156" t="inlineStr">
@@ -5148,12 +5148,12 @@
       </c>
       <c r="F156" t="inlineStr">
         <is>
-          <t>GO</t>
+          <t>EIFFAGE</t>
         </is>
       </c>
       <c r="G156" t="inlineStr">
         <is>
-          <t>DPGF GO 5.10.2 (m²). Contrôle à 1 mois / tonte à 15 j hors planning. | Durée recalée EXE (15 semaines) : renfort d'équipes / travail en parallèle.</t>
+          <t>DPGF EIFFAGE 5.10.2 (m²). Contrôle à 1 mois / tonte à 15 j hors planning. | Durée recalée EXE (15 semaines) : renfort d'équipes / travail en parallèle.</t>
         </is>
       </c>
     </row>
@@ -5166,7 +5166,7 @@
       </c>
       <c r="C157" t="inlineStr">
         <is>
-          <t>[VRD] Réfection des cheminements de chantier</t>
+          <t>[EIFFAGE] Réfection des cheminements de chantier</t>
         </is>
       </c>
       <c r="D157" t="inlineStr">
@@ -5181,7 +5181,7 @@
       </c>
       <c r="F157" t="inlineStr">
         <is>
-          <t>GO</t>
+          <t>EIFFAGE</t>
         </is>
       </c>
       <c r="G157" t="inlineStr">
@@ -5199,7 +5199,7 @@
       </c>
       <c r="C158" t="inlineStr">
         <is>
-          <t>[VRD] Curage + contrôle caméra des réseaux EU en fin de travaux</t>
+          <t>[EIFFAGE] Curage + contrôle caméra des réseaux EU en fin de travaux</t>
         </is>
       </c>
       <c r="D158" t="inlineStr">
@@ -5214,7 +5214,7 @@
       </c>
       <c r="F158" t="inlineStr">
         <is>
-          <t>GO</t>
+          <t>EIFFAGE</t>
         </is>
       </c>
       <c r="G158" t="inlineStr">
@@ -5245,7 +5245,7 @@
       </c>
       <c r="C160" t="inlineStr">
         <is>
-          <t>[GO] Constat d'huissier contradictoire de fin de travaux</t>
+          <t>[EIFFAGE] Constat d'huissier contradictoire de fin de travaux</t>
         </is>
       </c>
       <c r="D160" t="inlineStr">
@@ -5260,12 +5260,12 @@
       </c>
       <c r="F160" t="inlineStr">
         <is>
-          <t>GO</t>
+          <t>EIFFAGE</t>
         </is>
       </c>
       <c r="G160" t="inlineStr">
         <is>
-          <t>DPGF GO 5.1.1 ; CCTP GO 5.1.1.</t>
+          <t>DPGF EIFFAGE 5.1.1 ; CCTP EIFFAGE 5.1.1.</t>
         </is>
       </c>
     </row>
@@ -5278,7 +5278,7 @@
       </c>
       <c r="C161" t="inlineStr">
         <is>
-          <t>[GO] DOE lot GO/VRD : récolement ouvrages enterrés, PV essais béton/pieux, fiches techniques</t>
+          <t>[EIFFAGE] DOE lot EIFFAGE : récolement ouvrages enterrés, PV essais béton/pieux, fiches techniques</t>
         </is>
       </c>
       <c r="D161" t="inlineStr">
@@ -5293,12 +5293,12 @@
       </c>
       <c r="F161" t="inlineStr">
         <is>
-          <t>GO</t>
+          <t>EIFFAGE</t>
         </is>
       </c>
       <c r="G161" t="inlineStr">
         <is>
-          <t>Limites : DOE chacun pour son lot ; CCTP GO 2.3.7. | Durée recalée EXE (15 semaines) : renfort d'équipes / travail en parallèle.</t>
+          <t>Limites : DOE chacun pour son lot ; CCTP EIFFAGE 2.3.7. | Durée recalée EXE (15 semaines) : renfort d'équipes / travail en parallèle.</t>
         </is>
       </c>
     </row>
@@ -5419,7 +5419,7 @@
       </c>
       <c r="C166" t="inlineStr">
         <is>
-          <t>[GO] Gestion des portails / accès de chantier (ouverture, fermeture, surveillance)</t>
+          <t>[EIFFAGE] Gestion des portails / accès de chantier (ouverture, fermeture, surveillance)</t>
         </is>
       </c>
       <c r="D166" t="inlineStr">
@@ -5434,12 +5434,12 @@
       </c>
       <c r="F166" t="inlineStr">
         <is>
-          <t>GO</t>
+          <t>EIFFAGE</t>
         </is>
       </c>
       <c r="G166" t="inlineStr">
         <is>
-          <t>Limites de prestations 1 : GO phase 1 ; CCTP GO 5.1.3.</t>
+          <t>Limites de prestations 1 : EIFFAGE phase 1 ; CCTP EIFFAGE 5.1.3.</t>
         </is>
       </c>
     </row>
@@ -5452,7 +5452,7 @@
       </c>
       <c r="C167" t="inlineStr">
         <is>
-          <t>[GO] Entretien et nettoyage des abords, accès et voies (permanent)</t>
+          <t>[EIFFAGE] Entretien et nettoyage des abords, accès et voies (permanent)</t>
         </is>
       </c>
       <c r="D167" t="inlineStr">
@@ -5467,12 +5467,12 @@
       </c>
       <c r="F167" t="inlineStr">
         <is>
-          <t>GO</t>
+          <t>EIFFAGE</t>
         </is>
       </c>
       <c r="G167" t="inlineStr">
         <is>
-          <t>DPGF GO 5.1.11 ; CCTP GO 5.1.11.</t>
+          <t>DPGF EIFFAGE 5.1.11 ; CCTP EIFFAGE 5.1.11.</t>
         </is>
       </c>
     </row>
@@ -5485,7 +5485,7 @@
       </c>
       <c r="C168" t="inlineStr">
         <is>
-          <t>[GO/VRD] Homme trafic (voie pompier, arrivées/départs camions) - phases démolition à remise en état</t>
+          <t>[EIFFAGE] Homme trafic (voie pompier, arrivées/départs camions) - phases démolition à remise en état</t>
         </is>
       </c>
       <c r="D168" t="inlineStr">
@@ -5500,12 +5500,12 @@
       </c>
       <c r="F168" t="inlineStr">
         <is>
-          <t>GO</t>
+          <t>EIFFAGE</t>
         </is>
       </c>
       <c r="G168" t="inlineStr">
         <is>
-          <t>DPGF GO 5.1.12 ; Limites de prestations 2 (chacun pour son lot).</t>
+          <t>DPGF EIFFAGE 5.1.12 ; Limites de prestations 2 (chacun pour son lot).</t>
         </is>
       </c>
     </row>
@@ -5584,7 +5584,7 @@
       </c>
       <c r="C171" t="inlineStr">
         <is>
-          <t>[GO] Bennes de chantier + évacuation gravats (part du lot)</t>
+          <t>[EIFFAGE] Bennes de chantier + évacuation gravats (part du lot)</t>
         </is>
       </c>
       <c r="D171" t="inlineStr">
@@ -5599,12 +5599,12 @@
       </c>
       <c r="F171" t="inlineStr">
         <is>
-          <t>GO</t>
+          <t>EIFFAGE</t>
         </is>
       </c>
       <c r="G171" t="inlineStr">
         <is>
-          <t>DPGF GO 5.1.10.</t>
+          <t>DPGF EIFFAGE 5.1.10.</t>
         </is>
       </c>
     </row>

</xml_diff>